<commit_message>
feat: complete TechBots-SIT RFID attendance system with 6-section navigation, settings page, and 17 passing tests
</commit_message>
<xml_diff>
--- a/data/attendance_records.xlsx
+++ b/data/attendance_records.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -619,6 +619,43 @@
       <c r="G6" t="inlineStr">
         <is>
           <t>PRESENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ananya udupi</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>CSE</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>4SN25CS002</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>07:55 PM</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>08:02 PM</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Left</t>
         </is>
       </c>
     </row>

</xml_diff>